<commit_message>
correzione rates in rete classica
</commit_message>
<xml_diff>
--- a/Pipe_Matlab_Indici_di_Prestazione_Classica/FOLDER/EXCEL.xlsx
+++ b/Pipe_Matlab_Indici_di_Prestazione_Classica/FOLDER/EXCEL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lachiara\Desktop\Uni_Andrea\Magistrale\Secondo_Anno\Controllo_Avanzato\Pipe_Matlab\FOLDER\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lachiara\Documents\GitHub\ControlloAvanzato\Pipe_Matlab_Indici_di_Prestazione_Classica\FOLDER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2839A6D-5D6E-4EA9-95B5-8D14186EBE24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37895CE6-AA81-4256-99EA-15490F4DA94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="68">
   <si>
     <t>Petri net incidence and marking</t>
   </si>
@@ -290,6 +290,21 @@
   </si>
   <si>
     <t>descrizione</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1/2</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1/6</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1/5</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1/8</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1/3</t>
   </si>
 </sst>
 </file>
@@ -7975,7 +7990,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="135" spans="1:30" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:30" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="3" t="s">
         <v>2</v>
       </c>
@@ -8146,14 +8161,14 @@
       <c r="N139" s="7"/>
     </row>
     <row r="140" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A140">
-        <v>2</v>
-      </c>
-      <c r="B140">
-        <v>6</v>
-      </c>
-      <c r="C140">
-        <v>2</v>
+      <c r="A140" t="s">
+        <v>63</v>
+      </c>
+      <c r="B140" t="s">
+        <v>64</v>
+      </c>
+      <c r="C140" t="s">
+        <v>63</v>
       </c>
       <c r="D140">
         <v>0</v>
@@ -8167,35 +8182,35 @@
       <c r="G140">
         <v>0</v>
       </c>
-      <c r="H140">
-        <v>2</v>
-      </c>
-      <c r="I140">
-        <v>5</v>
-      </c>
-      <c r="J140">
-        <v>2</v>
+      <c r="H140" t="s">
+        <v>63</v>
+      </c>
+      <c r="I140" t="s">
+        <v>65</v>
+      </c>
+      <c r="J140" t="s">
+        <v>63</v>
       </c>
       <c r="K140">
         <v>0</v>
       </c>
-      <c r="L140">
-        <v>2</v>
-      </c>
-      <c r="M140">
-        <v>5</v>
-      </c>
-      <c r="N140" s="7">
-        <v>2</v>
+      <c r="L140" t="s">
+        <v>63</v>
+      </c>
+      <c r="M140" t="s">
+        <v>65</v>
+      </c>
+      <c r="N140" s="7" t="s">
+        <v>63</v>
       </c>
       <c r="O140">
         <v>0</v>
       </c>
-      <c r="P140">
-        <v>8</v>
-      </c>
-      <c r="Q140">
-        <v>3</v>
+      <c r="P140" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q140" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="141" spans="1:30" x14ac:dyDescent="0.3">

</xml_diff>